<commit_message>
docs: Synchronize updated INSTRUCTIONS.md and carga_masiva.xlsx
</commit_message>
<xml_diff>
--- a/carga_masiva.xlsx
+++ b/carga_masiva.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Mi unidad\Perico_ENJOY\Consola_Enjoy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B9C6308-EB5C-4C21-8F4B-A2AC3757792A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1D14408-A404-4FC3-B36D-1D5932F03E6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-888" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="tareas" sheetId="1" r:id="rId1"/>
     <sheet name="Hoja1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">tareas!$A$1:$R$62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">tareas!$A$1:$S$62</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="725" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="740" uniqueCount="244">
   <si>
     <t>id_proyecto</t>
   </si>
@@ -777,6 +777,9 @@
   </si>
   <si>
     <t>proyecto_descripcion</t>
+  </si>
+  <si>
+    <t>tarea_fecha_creacion</t>
   </si>
 </sst>
 </file>
@@ -857,7 +860,7 @@
     <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -877,7 +880,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1127,10 +1129,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:R62"/>
+  <dimension ref="A1:S62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="12.85546875" customWidth="1"/>
@@ -1141,18 +1143,19 @@
     <col min="7" max="7" width="14.28515625" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="96" customWidth="1"/>
     <col min="10" max="10" width="13.28515625" style="5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.28515625" style="19" customWidth="1"/>
-    <col min="12" max="12" width="13.28515625" style="16" customWidth="1"/>
-    <col min="13" max="13" width="13.140625" style="5" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="13.28515625" style="5" customWidth="1"/>
-    <col min="15" max="15" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="14.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="14.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.28515625" style="18" customWidth="1"/>
+    <col min="12" max="12" width="13.28515625" style="15" customWidth="1"/>
+    <col min="13" max="13" width="14.5703125" customWidth="1"/>
+    <col min="14" max="14" width="13.140625" style="5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.28515625" style="5" customWidth="1"/>
+    <col min="16" max="16" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="14.7109375" style="5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="14.140625" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="A1" s="9" t="s">
         <v>225</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1167,7 +1170,7 @@
       <c r="E1" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="F1" s="10" t="s">
+      <c r="F1" s="9" t="s">
         <v>226</v>
       </c>
       <c r="G1" s="1" t="s">
@@ -1176,38 +1179,41 @@
       <c r="H1" s="1" t="s">
         <v>149</v>
       </c>
-      <c r="I1" s="10" t="s">
+      <c r="I1" s="9" t="s">
         <v>224</v>
       </c>
       <c r="J1" s="6" t="s">
         <v>228</v>
       </c>
-      <c r="K1" s="17" t="s">
+      <c r="K1" s="16" t="s">
         <v>229</v>
       </c>
-      <c r="L1" s="14" t="s">
+      <c r="L1" s="13" t="s">
         <v>230</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="M1" s="9" t="s">
+        <v>243</v>
+      </c>
+      <c r="N1" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="N1" s="6" t="s">
+      <c r="O1" s="6" t="s">
         <v>219</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="S1" s="3" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
@@ -1230,32 +1236,35 @@
       <c r="H2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="I2" s="13" t="s">
+      <c r="I2" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J2" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="K2" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L2" s="15">
+      <c r="L2" s="14">
         <v>1</v>
       </c>
-      <c r="M2" s="4">
+      <c r="M2" s="19">
         <v>46198</v>
       </c>
-      <c r="N2" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q2" s="21">
+      <c r="N2" s="4">
         <v>46198</v>
       </c>
-      <c r="R2" s="21">
+      <c r="O2" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R2" s="20">
         <v>46198</v>
       </c>
-    </row>
-    <row r="3" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S2" s="20">
+        <v>46198</v>
+      </c>
+    </row>
+    <row r="3" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>6</v>
       </c>
@@ -1278,26 +1287,29 @@
       <c r="H3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I3" s="13" t="s">
+      <c r="I3" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J3" s="7" t="s">
         <v>214</v>
       </c>
-      <c r="K3" s="18" t="s">
+      <c r="K3" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L3" s="15"/>
-      <c r="M3" s="4" t="s">
+      <c r="L3" s="14"/>
+      <c r="M3" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N3" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q3"/>
+      <c r="N3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O3" s="7" t="s">
+        <v>220</v>
+      </c>
       <c r="R3"/>
-    </row>
-    <row r="4" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S3"/>
+    </row>
+    <row r="4" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
@@ -1320,32 +1332,35 @@
       <c r="H4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="13" t="s">
+      <c r="I4" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J4" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K4" s="18" t="s">
+      <c r="K4" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L4" s="15">
+      <c r="L4" s="14">
         <v>1</v>
       </c>
-      <c r="M4" s="4">
+      <c r="M4" s="19">
         <v>46226</v>
       </c>
-      <c r="N4" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q4" s="21">
+      <c r="N4" s="4">
         <v>46226</v>
       </c>
-      <c r="R4" s="21">
+      <c r="O4" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R4" s="20">
         <v>46226</v>
       </c>
-    </row>
-    <row r="5" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S4" s="20">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="5" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>6</v>
       </c>
@@ -1368,26 +1383,29 @@
       <c r="H5" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="I5" s="13" t="s">
+      <c r="I5" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J5" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K5" s="18" t="s">
+      <c r="K5" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L5" s="15"/>
-      <c r="M5" s="4" t="s">
+      <c r="L5" s="14"/>
+      <c r="M5" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N5" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q5"/>
+      <c r="N5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O5" s="7" t="s">
+        <v>220</v>
+      </c>
       <c r="R5"/>
-    </row>
-    <row r="6" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S5"/>
+    </row>
+    <row r="6" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
@@ -1410,26 +1428,29 @@
       <c r="H6" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="I6" s="13" t="s">
+      <c r="I6" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J6" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K6" s="18" t="s">
+      <c r="K6" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L6" s="15"/>
-      <c r="M6" s="4" t="s">
+      <c r="L6" s="14"/>
+      <c r="M6" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N6" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q6"/>
+      <c r="N6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O6" s="7" t="s">
+        <v>220</v>
+      </c>
       <c r="R6"/>
-    </row>
-    <row r="7" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S6"/>
+    </row>
+    <row r="7" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
         <v>6</v>
       </c>
@@ -1452,26 +1473,29 @@
       <c r="H7" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="I7" s="13" t="s">
+      <c r="I7" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J7" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K7" s="18" t="s">
+      <c r="K7" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L7" s="15"/>
-      <c r="M7" s="4" t="s">
+      <c r="L7" s="14"/>
+      <c r="M7" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N7" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q7"/>
+      <c r="N7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O7" s="7" t="s">
+        <v>220</v>
+      </c>
       <c r="R7"/>
-    </row>
-    <row r="8" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S7"/>
+    </row>
+    <row r="8" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>22</v>
       </c>
@@ -1491,35 +1515,38 @@
       <c r="G8" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="8" t="s">
         <v>216</v>
       </c>
-      <c r="I8" s="13" t="s">
+      <c r="I8" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J8" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K8" s="18" t="s">
+      <c r="K8" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L8" s="15">
+      <c r="L8" s="14">
         <v>1</v>
       </c>
-      <c r="M8" s="4">
+      <c r="M8" s="19">
         <v>46182</v>
       </c>
-      <c r="N8" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q8" s="21">
+      <c r="N8" s="4">
         <v>46182</v>
       </c>
-      <c r="R8" s="21">
+      <c r="O8" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R8" s="20">
         <v>46182</v>
       </c>
-    </row>
-    <row r="9" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S8" s="20">
+        <v>46182</v>
+      </c>
+    </row>
+    <row r="9" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>22</v>
       </c>
@@ -1542,32 +1569,35 @@
       <c r="H9" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="I9" s="13" t="s">
+      <c r="I9" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J9" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K9" s="18" t="s">
+      <c r="K9" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L9" s="15">
+      <c r="L9" s="14">
         <v>1</v>
       </c>
-      <c r="M9" s="4">
+      <c r="M9" s="19">
         <v>46192</v>
       </c>
-      <c r="N9" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q9" s="21">
+      <c r="N9" s="4">
         <v>46192</v>
       </c>
-      <c r="R9" s="21">
+      <c r="O9" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R9" s="20">
         <v>46192</v>
       </c>
-    </row>
-    <row r="10" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S9" s="20">
+        <v>46192</v>
+      </c>
+    </row>
+    <row r="10" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>22</v>
       </c>
@@ -1590,32 +1620,35 @@
       <c r="H10" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="I10" s="13" t="s">
+      <c r="I10" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J10" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K10" s="18" t="s">
+      <c r="K10" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L10" s="15">
+      <c r="L10" s="14">
         <v>1</v>
       </c>
-      <c r="M10" s="4">
+      <c r="M10" s="19">
         <v>46197</v>
       </c>
-      <c r="N10" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q10" s="21">
+      <c r="N10" s="4">
         <v>46197</v>
       </c>
-      <c r="R10" s="21">
+      <c r="O10" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R10" s="20">
         <v>46197</v>
       </c>
-    </row>
-    <row r="11" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S10" s="20">
+        <v>46197</v>
+      </c>
+    </row>
+    <row r="11" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>22</v>
       </c>
@@ -1638,32 +1671,35 @@
       <c r="H11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="I11" s="13" t="s">
+      <c r="I11" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J11" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K11" s="18" t="s">
+      <c r="K11" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L11" s="15">
+      <c r="L11" s="14">
         <v>1</v>
       </c>
-      <c r="M11" s="4">
+      <c r="M11" s="19">
         <v>46198</v>
       </c>
-      <c r="N11" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q11" s="21">
+      <c r="N11" s="4">
         <v>46198</v>
       </c>
-      <c r="R11" s="21">
+      <c r="O11" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R11" s="20">
         <v>46198</v>
       </c>
-    </row>
-    <row r="12" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S11" s="20">
+        <v>46198</v>
+      </c>
+    </row>
+    <row r="12" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>22</v>
       </c>
@@ -1686,32 +1722,35 @@
       <c r="H12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="I12" s="13" t="s">
+      <c r="I12" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J12" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K12" s="18" t="s">
+      <c r="K12" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L12" s="15">
+      <c r="L12" s="14">
         <v>1</v>
       </c>
-      <c r="M12" s="4">
+      <c r="M12" s="19">
         <v>46205</v>
       </c>
-      <c r="N12" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q12" s="21">
+      <c r="N12" s="4">
         <v>46205</v>
       </c>
-      <c r="R12" s="21">
+      <c r="O12" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R12" s="20">
         <v>46205</v>
       </c>
-    </row>
-    <row r="13" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S12" s="20">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="13" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>22</v>
       </c>
@@ -1734,32 +1773,35 @@
       <c r="H13" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="I13" s="13" t="s">
+      <c r="I13" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J13" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K13" s="18" t="s">
+      <c r="K13" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L13" s="15">
+      <c r="L13" s="14">
         <v>1</v>
       </c>
-      <c r="M13" s="4">
+      <c r="M13" s="19">
         <v>46205</v>
       </c>
-      <c r="N13" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q13" s="21">
+      <c r="N13" s="4">
         <v>46205</v>
       </c>
-      <c r="R13" s="21">
+      <c r="O13" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R13" s="20">
         <v>46205</v>
       </c>
-    </row>
-    <row r="14" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S13" s="20">
+        <v>46205</v>
+      </c>
+    </row>
+    <row r="14" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>22</v>
       </c>
@@ -1782,32 +1824,35 @@
       <c r="H14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="I14" s="13" t="s">
+      <c r="I14" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J14" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K14" s="18" t="s">
+      <c r="K14" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L14" s="15">
+      <c r="L14" s="14">
         <v>1</v>
       </c>
-      <c r="M14" s="4">
+      <c r="M14" s="19">
         <v>46211</v>
       </c>
-      <c r="N14" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q14" s="21">
+      <c r="N14" s="4">
         <v>46211</v>
       </c>
-      <c r="R14" s="21">
+      <c r="O14" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R14" s="20">
         <v>46211</v>
       </c>
-    </row>
-    <row r="15" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S14" s="20">
+        <v>46211</v>
+      </c>
+    </row>
+    <row r="15" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>22</v>
       </c>
@@ -1830,32 +1875,35 @@
       <c r="H15" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="I15" s="13" t="s">
+      <c r="I15" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J15" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K15" s="18" t="s">
+      <c r="K15" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L15" s="15"/>
-      <c r="M15" s="4">
+      <c r="L15" s="14"/>
+      <c r="M15" s="19">
         <v>46213</v>
       </c>
-      <c r="N15" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="O15" s="20">
+      <c r="N15" s="4">
         <v>46213</v>
       </c>
-      <c r="P15" s="20">
+      <c r="O15" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="P15" s="19">
         <v>46213</v>
       </c>
-      <c r="Q15"/>
+      <c r="Q15" s="19">
+        <v>46213</v>
+      </c>
       <c r="R15"/>
-    </row>
-    <row r="16" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S15"/>
+    </row>
+    <row r="16" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A16" s="2" t="s">
         <v>22</v>
       </c>
@@ -1878,32 +1926,35 @@
       <c r="H16" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="I16" s="13" t="s">
+      <c r="I16" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J16" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K16" s="18" t="s">
+      <c r="K16" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L16" s="15">
+      <c r="L16" s="14">
         <v>1</v>
       </c>
-      <c r="M16" s="4">
+      <c r="M16" s="19">
         <v>46216</v>
       </c>
-      <c r="N16" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q16" s="21">
+      <c r="N16" s="4">
         <v>46216</v>
       </c>
-      <c r="R16" s="21">
+      <c r="O16" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R16" s="20">
         <v>46216</v>
       </c>
-    </row>
-    <row r="17" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S16" s="20">
+        <v>46216</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>22</v>
       </c>
@@ -1926,32 +1977,35 @@
       <c r="H17" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="I17" s="13" t="s">
+      <c r="I17" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J17" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K17" s="18" t="s">
+      <c r="K17" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L17" s="15">
+      <c r="L17" s="14">
         <v>1</v>
       </c>
-      <c r="M17" s="4">
+      <c r="M17" s="19">
         <v>46218</v>
       </c>
-      <c r="N17" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q17" s="21">
+      <c r="N17" s="4">
         <v>46218</v>
       </c>
-      <c r="R17" s="21">
+      <c r="O17" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R17" s="20">
         <v>46218</v>
       </c>
-    </row>
-    <row r="18" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S17" s="20">
+        <v>46218</v>
+      </c>
+    </row>
+    <row r="18" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A18" s="2" t="s">
         <v>22</v>
       </c>
@@ -1974,32 +2028,35 @@
       <c r="H18" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="I18" s="13" t="s">
+      <c r="I18" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J18" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K18" s="18" t="s">
+      <c r="K18" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L18" s="15">
+      <c r="L18" s="14">
         <v>1</v>
       </c>
-      <c r="M18" s="4">
+      <c r="M18" s="19">
         <v>46225</v>
       </c>
-      <c r="N18" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q18" s="21">
+      <c r="N18" s="4">
         <v>46225</v>
       </c>
-      <c r="R18" s="21">
+      <c r="O18" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R18" s="20">
         <v>46225</v>
       </c>
-    </row>
-    <row r="19" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S18" s="20">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>22</v>
       </c>
@@ -2022,32 +2079,35 @@
       <c r="H19" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="I19" s="13" t="s">
+      <c r="I19" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J19" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K19" s="18" t="s">
+      <c r="K19" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L19" s="15">
+      <c r="L19" s="14">
         <v>1</v>
       </c>
-      <c r="M19" s="4">
+      <c r="M19" s="19">
         <v>46226</v>
       </c>
-      <c r="N19" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q19" s="21">
+      <c r="N19" s="4">
         <v>46226</v>
       </c>
-      <c r="R19" s="21">
+      <c r="O19" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R19" s="20">
         <v>46226</v>
       </c>
-    </row>
-    <row r="20" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S19" s="20">
+        <v>46226</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>47</v>
       </c>
@@ -2067,35 +2127,38 @@
       <c r="G20" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="H20" s="9" t="s">
+      <c r="H20" s="8" t="s">
         <v>217</v>
       </c>
-      <c r="I20" s="13" t="s">
+      <c r="I20" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J20" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K20" s="18" t="s">
+      <c r="K20" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L20" s="15"/>
-      <c r="M20" s="4">
+      <c r="L20" s="14"/>
+      <c r="M20" s="19">
         <v>46190</v>
       </c>
-      <c r="N20" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="O20" s="20">
+      <c r="N20" s="4">
         <v>46190</v>
       </c>
-      <c r="P20" s="20">
+      <c r="O20" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="P20" s="19">
         <v>46190</v>
       </c>
-      <c r="Q20"/>
+      <c r="Q20" s="19">
+        <v>46190</v>
+      </c>
       <c r="R20"/>
-    </row>
-    <row r="21" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S20"/>
+    </row>
+    <row r="21" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>47</v>
       </c>
@@ -2118,32 +2181,35 @@
       <c r="H21" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="I21" s="13" t="s">
+      <c r="I21" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J21" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K21" s="18" t="s">
+      <c r="K21" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L21" s="15"/>
-      <c r="M21" s="4">
+      <c r="L21" s="14"/>
+      <c r="M21" s="19">
         <v>46197</v>
       </c>
-      <c r="N21" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="O21" s="20">
+      <c r="N21" s="4">
         <v>46197</v>
       </c>
-      <c r="P21" s="20">
+      <c r="O21" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="P21" s="19">
         <v>46197</v>
       </c>
-      <c r="Q21"/>
+      <c r="Q21" s="19">
+        <v>46197</v>
+      </c>
       <c r="R21"/>
-    </row>
-    <row r="22" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S21"/>
+    </row>
+    <row r="22" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>47</v>
       </c>
@@ -2166,32 +2232,35 @@
       <c r="H22" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="I22" s="13" t="s">
+      <c r="I22" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J22" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K22" s="18" t="s">
+      <c r="K22" s="17" t="s">
         <v>238</v>
       </c>
-      <c r="L22" s="15"/>
-      <c r="M22" s="4">
+      <c r="L22" s="14"/>
+      <c r="M22" s="19">
         <v>46213</v>
       </c>
-      <c r="N22" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="O22" s="20">
+      <c r="N22" s="4">
         <v>46213</v>
       </c>
-      <c r="P22" s="20">
+      <c r="O22" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="P22" s="19">
         <v>46213</v>
       </c>
-      <c r="Q22"/>
+      <c r="Q22" s="19">
+        <v>46213</v>
+      </c>
       <c r="R22"/>
-    </row>
-    <row r="23" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S22"/>
+    </row>
+    <row r="23" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>47</v>
       </c>
@@ -2214,32 +2283,35 @@
       <c r="H23" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="I23" s="13" t="s">
+      <c r="I23" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J23" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K23" s="18" t="s">
+      <c r="K23" s="17" t="s">
         <v>238</v>
       </c>
-      <c r="L23" s="15"/>
-      <c r="M23" s="4">
+      <c r="L23" s="14"/>
+      <c r="M23" s="19">
         <v>46217</v>
       </c>
-      <c r="N23" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="O23" s="20">
+      <c r="N23" s="4">
         <v>46217</v>
       </c>
-      <c r="P23" s="20">
+      <c r="O23" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="P23" s="19">
         <v>46217</v>
       </c>
-      <c r="Q23"/>
+      <c r="Q23" s="19">
+        <v>46217</v>
+      </c>
       <c r="R23"/>
-    </row>
-    <row r="24" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S23"/>
+    </row>
+    <row r="24" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>47</v>
       </c>
@@ -2262,32 +2334,35 @@
       <c r="H24" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="I24" s="13" t="s">
+      <c r="I24" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J24" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K24" s="18" t="s">
+      <c r="K24" s="17" t="s">
         <v>238</v>
       </c>
-      <c r="L24" s="15"/>
-      <c r="M24" s="4">
+      <c r="L24" s="14"/>
+      <c r="M24" s="19">
         <v>46225</v>
       </c>
-      <c r="N24" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="O24" s="20">
+      <c r="N24" s="4">
         <v>46225</v>
       </c>
-      <c r="P24" s="20">
+      <c r="O24" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="P24" s="19">
         <v>46225</v>
       </c>
-      <c r="Q24"/>
+      <c r="Q24" s="19">
+        <v>46225</v>
+      </c>
       <c r="R24"/>
-    </row>
-    <row r="25" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S24"/>
+    </row>
+    <row r="25" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>47</v>
       </c>
@@ -2310,28 +2385,31 @@
       <c r="H25" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="I25" s="13" t="s">
+      <c r="I25" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J25" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K25" s="18" t="s">
+      <c r="K25" s="17" t="s">
         <v>238</v>
       </c>
-      <c r="L25" s="15">
+      <c r="L25" s="14">
         <v>1</v>
       </c>
-      <c r="M25" s="4" t="s">
+      <c r="M25" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N25" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q25"/>
+      <c r="N25" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O25" s="7" t="s">
+        <v>220</v>
+      </c>
       <c r="R25"/>
-    </row>
-    <row r="26" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S25"/>
+    </row>
+    <row r="26" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>47</v>
       </c>
@@ -2354,28 +2432,31 @@
       <c r="H26" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="I26" s="13" t="s">
+      <c r="I26" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J26" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K26" s="18" t="s">
+      <c r="K26" s="17" t="s">
         <v>238</v>
       </c>
-      <c r="L26" s="15">
+      <c r="L26" s="14">
         <v>1</v>
       </c>
-      <c r="M26" s="4" t="s">
+      <c r="M26" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N26" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q26"/>
+      <c r="N26" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O26" s="7" t="s">
+        <v>220</v>
+      </c>
       <c r="R26"/>
-    </row>
-    <row r="27" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S26"/>
+    </row>
+    <row r="27" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>47</v>
       </c>
@@ -2398,32 +2479,35 @@
       <c r="H27" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="I27" s="13" t="s">
+      <c r="I27" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J27" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K27" s="18" t="s">
+      <c r="K27" s="17" t="s">
         <v>238</v>
       </c>
-      <c r="L27" s="15">
+      <c r="L27" s="14">
         <v>1</v>
       </c>
-      <c r="M27" s="4">
+      <c r="M27" s="19">
         <v>46225</v>
       </c>
-      <c r="N27" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q27" s="21">
+      <c r="N27" s="4">
         <v>46225</v>
       </c>
-      <c r="R27" s="21">
+      <c r="O27" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R27" s="20">
         <v>46225</v>
       </c>
-    </row>
-    <row r="28" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S27" s="20">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="28" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>64</v>
       </c>
@@ -2446,26 +2530,29 @@
       <c r="H28" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="I28" s="13" t="s">
+      <c r="I28" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J28" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K28" s="18" t="s">
+      <c r="K28" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="L28" s="15"/>
-      <c r="M28" s="4" t="s">
+      <c r="L28" s="14"/>
+      <c r="M28" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N28" s="7" t="s">
+      <c r="N28" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O28" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="Q28"/>
       <c r="R28"/>
-    </row>
-    <row r="29" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S28"/>
+    </row>
+    <row r="29" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>64</v>
       </c>
@@ -2485,29 +2572,32 @@
       <c r="G29" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="H29" s="9" t="s">
+      <c r="H29" s="8" t="s">
         <v>218</v>
       </c>
-      <c r="I29" s="13" t="s">
+      <c r="I29" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J29" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K29" s="18" t="s">
+      <c r="K29" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="L29" s="15"/>
-      <c r="M29" s="4" t="s">
+      <c r="L29" s="14"/>
+      <c r="M29" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N29" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q29"/>
+      <c r="N29" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O29" s="7" t="s">
+        <v>220</v>
+      </c>
       <c r="R29"/>
-    </row>
-    <row r="30" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S29"/>
+    </row>
+    <row r="30" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>64</v>
       </c>
@@ -2530,32 +2620,35 @@
       <c r="H30" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="I30" s="13" t="s">
+      <c r="I30" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J30" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K30" s="18" t="s">
+      <c r="K30" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="L30" s="15">
+      <c r="L30" s="14">
         <v>1</v>
       </c>
-      <c r="M30" s="4">
+      <c r="M30" s="19">
         <v>46217</v>
       </c>
-      <c r="N30" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q30" s="21">
+      <c r="N30" s="4">
         <v>46217</v>
       </c>
-      <c r="R30" s="21">
+      <c r="O30" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R30" s="20">
         <v>46217</v>
       </c>
-    </row>
-    <row r="31" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S30" s="20">
+        <v>46217</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A31" s="2" t="s">
         <v>64</v>
       </c>
@@ -2578,26 +2671,29 @@
       <c r="H31" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="I31" s="13" t="s">
+      <c r="I31" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J31" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K31" s="18" t="s">
+      <c r="K31" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="L31" s="15"/>
-      <c r="M31" s="4" t="s">
+      <c r="L31" s="14"/>
+      <c r="M31" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N31" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q31"/>
+      <c r="N31" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O31" s="7" t="s">
+        <v>220</v>
+      </c>
       <c r="R31"/>
-    </row>
-    <row r="32" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S31"/>
+    </row>
+    <row r="32" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>64</v>
       </c>
@@ -2620,28 +2716,31 @@
       <c r="H32" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="I32" s="13" t="s">
+      <c r="I32" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J32" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K32" s="18" t="s">
+      <c r="K32" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="L32" s="15">
+      <c r="L32" s="14">
         <v>1</v>
       </c>
-      <c r="M32" s="4" t="s">
+      <c r="M32" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N32" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q32"/>
+      <c r="N32" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O32" s="7" t="s">
+        <v>220</v>
+      </c>
       <c r="R32"/>
-    </row>
-    <row r="33" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S32"/>
+    </row>
+    <row r="33" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>64</v>
       </c>
@@ -2664,28 +2763,31 @@
       <c r="H33" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="I33" s="13" t="s">
+      <c r="I33" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J33" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K33" s="18" t="s">
+      <c r="K33" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="L33" s="15">
+      <c r="L33" s="14">
         <v>1</v>
       </c>
-      <c r="M33" s="4" t="s">
+      <c r="M33" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N33" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q33"/>
+      <c r="N33" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O33" s="7" t="s">
+        <v>220</v>
+      </c>
       <c r="R33"/>
-    </row>
-    <row r="34" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S33"/>
+    </row>
+    <row r="34" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>64</v>
       </c>
@@ -2708,26 +2810,29 @@
       <c r="H34" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="I34" s="13" t="s">
+      <c r="I34" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J34" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K34" s="18" t="s">
+      <c r="K34" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="L34" s="15"/>
-      <c r="M34" s="4" t="s">
+      <c r="L34" s="14"/>
+      <c r="M34" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N34" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q34"/>
+      <c r="N34" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O34" s="7" t="s">
+        <v>220</v>
+      </c>
       <c r="R34"/>
-    </row>
-    <row r="35" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S34"/>
+    </row>
+    <row r="35" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>64</v>
       </c>
@@ -2750,32 +2855,35 @@
       <c r="H35" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="I35" s="13" t="s">
+      <c r="I35" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J35" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K35" s="18" t="s">
+      <c r="K35" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="L35" s="15">
+      <c r="L35" s="14">
         <v>1</v>
       </c>
-      <c r="M35" s="4">
+      <c r="M35" s="19">
         <v>46223</v>
       </c>
-      <c r="N35" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q35" s="21">
+      <c r="N35" s="4">
         <v>46223</v>
       </c>
-      <c r="R35" s="21">
+      <c r="O35" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R35" s="20">
         <v>46223</v>
       </c>
-    </row>
-    <row r="36" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S35" s="20">
+        <v>46223</v>
+      </c>
+    </row>
+    <row r="36" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>64</v>
       </c>
@@ -2798,32 +2906,35 @@
       <c r="H36" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="I36" s="13" t="s">
+      <c r="I36" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J36" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K36" s="18" t="s">
+      <c r="K36" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="L36" s="15"/>
-      <c r="M36" s="4">
+      <c r="L36" s="14"/>
+      <c r="M36" s="19">
         <v>46225</v>
       </c>
-      <c r="N36" s="7" t="s">
+      <c r="N36" s="4">
+        <v>46225</v>
+      </c>
+      <c r="O36" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="O36" s="20">
+      <c r="P36" s="19">
         <v>46225</v>
       </c>
-      <c r="P36" s="20">
+      <c r="Q36" s="19">
         <v>46225</v>
       </c>
-      <c r="Q36"/>
       <c r="R36"/>
-    </row>
-    <row r="37" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S36"/>
+    </row>
+    <row r="37" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>64</v>
       </c>
@@ -2846,32 +2957,35 @@
       <c r="H37" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="I37" s="13" t="s">
+      <c r="I37" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J37" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K37" s="18" t="s">
+      <c r="K37" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="L37" s="15">
+      <c r="L37" s="14">
         <v>1</v>
       </c>
-      <c r="M37" s="4">
+      <c r="M37" s="19">
         <v>46225</v>
       </c>
-      <c r="N37" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q37" s="21">
+      <c r="N37" s="4">
         <v>46225</v>
       </c>
-      <c r="R37" s="21">
+      <c r="O37" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R37" s="20">
         <v>46225</v>
       </c>
-    </row>
-    <row r="38" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S37" s="20">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="38" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>64</v>
       </c>
@@ -2894,32 +3008,35 @@
       <c r="H38" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="I38" s="13" t="s">
+      <c r="I38" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J38" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K38" s="18" t="s">
+      <c r="K38" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="L38" s="15"/>
-      <c r="M38" s="4">
+      <c r="L38" s="14"/>
+      <c r="M38" s="19">
         <v>46226</v>
       </c>
-      <c r="N38" s="7" t="s">
+      <c r="N38" s="4">
+        <v>46226</v>
+      </c>
+      <c r="O38" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="O38" s="20">
+      <c r="P38" s="19">
         <v>46226</v>
       </c>
-      <c r="P38" s="20">
+      <c r="Q38" s="19">
         <v>46226</v>
       </c>
-      <c r="Q38"/>
       <c r="R38"/>
-    </row>
-    <row r="39" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S38"/>
+    </row>
+    <row r="39" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>64</v>
       </c>
@@ -2942,32 +3059,35 @@
       <c r="H39" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I39" s="13" t="s">
+      <c r="I39" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J39" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K39" s="18" t="s">
+      <c r="K39" s="17" t="s">
         <v>239</v>
       </c>
-      <c r="L39" s="15">
+      <c r="L39" s="14">
         <v>1</v>
       </c>
-      <c r="M39" s="4">
+      <c r="M39" s="19">
         <v>46227</v>
       </c>
-      <c r="N39" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q39" s="21">
+      <c r="N39" s="4">
         <v>46227</v>
       </c>
-      <c r="R39" s="21">
+      <c r="O39" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R39" s="20">
         <v>46227</v>
       </c>
-    </row>
-    <row r="40" spans="1:18" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="S39" s="20">
+        <v>46227</v>
+      </c>
+    </row>
+    <row r="40" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>89</v>
       </c>
@@ -2990,26 +3110,29 @@
       <c r="H40" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="I40" s="13" t="s">
+      <c r="I40" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J40" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K40" s="18" t="s">
+      <c r="K40" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="L40" s="15"/>
-      <c r="M40" s="4" t="s">
+      <c r="L40" s="14"/>
+      <c r="M40" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N40" s="7" t="s">
+      <c r="N40" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O40" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="Q40"/>
       <c r="R40"/>
-    </row>
-    <row r="41" spans="1:18" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="S40"/>
+    </row>
+    <row r="41" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>89</v>
       </c>
@@ -3032,32 +3155,35 @@
       <c r="H41" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="I41" s="13" t="s">
+      <c r="I41" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J41" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K41" s="18" t="s">
+      <c r="K41" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="L41" s="15">
+      <c r="L41" s="14">
         <v>1</v>
       </c>
-      <c r="M41" s="4">
+      <c r="M41" s="19">
         <v>46049</v>
       </c>
-      <c r="N41" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q41" s="21">
+      <c r="N41" s="4">
         <v>46049</v>
       </c>
-      <c r="R41" s="21">
+      <c r="O41" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R41" s="20">
         <v>46049</v>
       </c>
-    </row>
-    <row r="42" spans="1:18" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="S41" s="20">
+        <v>46049</v>
+      </c>
+    </row>
+    <row r="42" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A42" s="2" t="s">
         <v>89</v>
       </c>
@@ -3080,32 +3206,35 @@
       <c r="H42" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="I42" s="13" t="s">
+      <c r="I42" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J42" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K42" s="18" t="s">
+      <c r="K42" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="L42" s="15">
+      <c r="L42" s="14">
         <v>1</v>
       </c>
-      <c r="M42" s="4">
+      <c r="M42" s="19">
         <v>46122</v>
       </c>
-      <c r="N42" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q42" s="21">
+      <c r="N42" s="4">
         <v>46122</v>
       </c>
-      <c r="R42" s="21">
+      <c r="O42" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R42" s="20">
         <v>46122</v>
       </c>
-    </row>
-    <row r="43" spans="1:18" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="S42" s="20">
+        <v>46122</v>
+      </c>
+    </row>
+    <row r="43" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>89</v>
       </c>
@@ -3128,26 +3257,29 @@
       <c r="H43" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="I43" s="13" t="s">
+      <c r="I43" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J43" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K43" s="18" t="s">
+      <c r="K43" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="L43" s="15"/>
-      <c r="M43" s="4" t="s">
+      <c r="L43" s="14"/>
+      <c r="M43" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="N43" s="7" t="s">
+      <c r="N43" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="O43" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="Q43"/>
       <c r="R43"/>
-    </row>
-    <row r="44" spans="1:18" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="S43"/>
+    </row>
+    <row r="44" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>89</v>
       </c>
@@ -3170,32 +3302,35 @@
       <c r="H44" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="I44" s="13" t="s">
+      <c r="I44" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J44" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K44" s="18" t="s">
+      <c r="K44" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="L44" s="15"/>
-      <c r="M44" s="4">
+      <c r="L44" s="14"/>
+      <c r="M44" s="19">
         <v>46209</v>
       </c>
-      <c r="N44" s="7" t="s">
+      <c r="N44" s="4">
+        <v>46209</v>
+      </c>
+      <c r="O44" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="O44" s="20">
+      <c r="P44" s="19">
         <v>46209</v>
       </c>
-      <c r="P44" s="20">
+      <c r="Q44" s="19">
         <v>46209</v>
       </c>
-      <c r="Q44"/>
       <c r="R44"/>
-    </row>
-    <row r="45" spans="1:18" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="S44"/>
+    </row>
+    <row r="45" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>89</v>
       </c>
@@ -3218,32 +3353,35 @@
       <c r="H45" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="I45" s="13" t="s">
+      <c r="I45" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J45" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K45" s="18" t="s">
+      <c r="K45" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="L45" s="15">
+      <c r="L45" s="14">
         <v>1</v>
       </c>
-      <c r="M45" s="4">
+      <c r="M45" s="19">
         <v>46213</v>
       </c>
-      <c r="N45" s="7" t="s">
+      <c r="N45" s="4">
+        <v>46213</v>
+      </c>
+      <c r="O45" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="Q45" s="21">
+      <c r="R45" s="20">
         <v>46213</v>
       </c>
-      <c r="R45" s="21">
+      <c r="S45" s="20">
         <v>46213</v>
       </c>
     </row>
-    <row r="46" spans="1:18" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>89</v>
       </c>
@@ -3266,32 +3404,35 @@
       <c r="H46" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="I46" s="13" t="s">
+      <c r="I46" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J46" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K46" s="18" t="s">
+      <c r="K46" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="L46" s="15">
+      <c r="L46" s="14">
         <v>1</v>
       </c>
-      <c r="M46" s="4">
+      <c r="M46" s="19">
         <v>46227</v>
       </c>
-      <c r="N46" s="7" t="s">
+      <c r="N46" s="4">
+        <v>46227</v>
+      </c>
+      <c r="O46" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="Q46" s="21">
+      <c r="R46" s="20">
         <v>46227</v>
       </c>
-      <c r="R46" s="21">
+      <c r="S46" s="20">
         <v>46227</v>
       </c>
     </row>
-    <row r="47" spans="1:18" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>89</v>
       </c>
@@ -3314,32 +3455,35 @@
       <c r="H47" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="I47" s="13" t="s">
+      <c r="I47" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J47" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K47" s="18" t="s">
+      <c r="K47" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="L47" s="15"/>
-      <c r="M47" s="4">
+      <c r="L47" s="14"/>
+      <c r="M47" s="19">
         <v>46213</v>
       </c>
-      <c r="N47" s="7" t="s">
+      <c r="N47" s="4">
+        <v>46213</v>
+      </c>
+      <c r="O47" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="O47" s="20">
+      <c r="P47" s="19">
         <v>46213</v>
       </c>
-      <c r="P47" s="20">
+      <c r="Q47" s="19">
         <v>46213</v>
       </c>
-      <c r="Q47"/>
       <c r="R47"/>
-    </row>
-    <row r="48" spans="1:18" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="S47"/>
+    </row>
+    <row r="48" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>89</v>
       </c>
@@ -3362,32 +3506,35 @@
       <c r="H48" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="I48" s="13" t="s">
+      <c r="I48" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J48" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K48" s="18" t="s">
+      <c r="K48" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="L48" s="15">
+      <c r="L48" s="14">
         <v>1</v>
       </c>
-      <c r="M48" s="4">
+      <c r="M48" s="19">
         <v>46223</v>
       </c>
-      <c r="N48" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q48" s="21">
+      <c r="N48" s="4">
         <v>46223</v>
       </c>
-      <c r="R48" s="21">
+      <c r="O48" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R48" s="20">
         <v>46223</v>
       </c>
-    </row>
-    <row r="49" spans="1:18" ht="12.75" x14ac:dyDescent="0.2">
+      <c r="S48" s="20">
+        <v>46223</v>
+      </c>
+    </row>
+    <row r="49" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>89</v>
       </c>
@@ -3410,32 +3557,35 @@
       <c r="H49" s="2" t="s">
         <v>112</v>
       </c>
-      <c r="I49" s="13" t="s">
+      <c r="I49" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J49" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K49" s="18" t="s">
+      <c r="K49" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="L49" s="15">
+      <c r="L49" s="14">
         <v>1</v>
       </c>
-      <c r="M49" s="4">
+      <c r="M49" s="19">
         <v>46225</v>
       </c>
-      <c r="N49" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q49" s="21">
+      <c r="N49" s="4">
         <v>46225</v>
       </c>
-      <c r="R49" s="21">
+      <c r="O49" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R49" s="20">
         <v>46225</v>
       </c>
-    </row>
-    <row r="50" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S49" s="20">
+        <v>46225</v>
+      </c>
+    </row>
+    <row r="50" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>113</v>
       </c>
@@ -3458,32 +3608,35 @@
       <c r="H50" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="I50" s="13" t="s">
+      <c r="I50" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J50" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K50" s="18" t="s">
+      <c r="K50" s="17" t="s">
         <v>241</v>
       </c>
-      <c r="L50" s="15"/>
-      <c r="M50" s="4">
+      <c r="L50" s="14"/>
+      <c r="M50" s="19">
         <v>45933</v>
       </c>
-      <c r="N50" s="7" t="s">
+      <c r="N50" s="4">
+        <v>45933</v>
+      </c>
+      <c r="O50" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="O50" s="20">
+      <c r="P50" s="19">
         <v>45933</v>
       </c>
-      <c r="P50" s="20">
+      <c r="Q50" s="19">
         <v>45933</v>
       </c>
-      <c r="Q50"/>
       <c r="R50"/>
-    </row>
-    <row r="51" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S50"/>
+    </row>
+    <row r="51" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>113</v>
       </c>
@@ -3506,32 +3659,35 @@
       <c r="H51" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="I51" s="13" t="s">
+      <c r="I51" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J51" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K51" s="18" t="s">
+      <c r="K51" s="17" t="s">
         <v>241</v>
       </c>
-      <c r="L51" s="15">
+      <c r="L51" s="14">
         <v>1</v>
       </c>
-      <c r="M51" s="4">
+      <c r="M51" s="19">
         <v>45950</v>
       </c>
-      <c r="N51" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q51" s="21">
+      <c r="N51" s="4">
         <v>45950</v>
       </c>
-      <c r="R51" s="21">
+      <c r="O51" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R51" s="20">
         <v>45950</v>
       </c>
-    </row>
-    <row r="52" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S51" s="20">
+        <v>45950</v>
+      </c>
+    </row>
+    <row r="52" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>113</v>
       </c>
@@ -3554,32 +3710,35 @@
       <c r="H52" s="8" t="s">
         <v>222</v>
       </c>
-      <c r="I52" s="13" t="s">
+      <c r="I52" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J52" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K52" s="18" t="s">
+      <c r="K52" s="17" t="s">
         <v>241</v>
       </c>
-      <c r="L52" s="15">
+      <c r="L52" s="14">
         <v>1</v>
       </c>
-      <c r="M52" s="4">
+      <c r="M52" s="19">
         <v>45982</v>
       </c>
-      <c r="N52" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q52" s="21">
+      <c r="N52" s="4">
         <v>45982</v>
       </c>
-      <c r="R52" s="21">
+      <c r="O52" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R52" s="20">
         <v>45982</v>
       </c>
-    </row>
-    <row r="53" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S52" s="20">
+        <v>45982</v>
+      </c>
+    </row>
+    <row r="53" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>113</v>
       </c>
@@ -3602,32 +3761,35 @@
       <c r="H53" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="I53" s="13" t="s">
+      <c r="I53" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J53" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="K53" s="18" t="s">
+      <c r="K53" s="17" t="s">
         <v>241</v>
       </c>
-      <c r="L53" s="15">
+      <c r="L53" s="14">
         <v>1</v>
       </c>
-      <c r="M53" s="4">
+      <c r="M53" s="19">
         <v>46008</v>
       </c>
-      <c r="N53" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="Q53" s="21">
+      <c r="N53" s="4">
         <v>46008</v>
       </c>
-      <c r="R53" s="21">
+      <c r="O53" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="R53" s="20">
         <v>46008</v>
       </c>
-    </row>
-    <row r="54" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S53" s="20">
+        <v>46008</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>113</v>
       </c>
@@ -3650,32 +3812,35 @@
       <c r="H54" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="I54" s="13" t="s">
+      <c r="I54" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J54" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K54" s="18" t="s">
+      <c r="K54" s="17" t="s">
         <v>241</v>
       </c>
-      <c r="L54" s="15"/>
-      <c r="M54" s="4">
+      <c r="L54" s="14"/>
+      <c r="M54" s="19">
         <v>46030</v>
       </c>
-      <c r="N54" s="7" t="s">
+      <c r="N54" s="4">
+        <v>46030</v>
+      </c>
+      <c r="O54" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="O54" s="20">
+      <c r="P54" s="19">
         <v>46030</v>
       </c>
-      <c r="P54" s="20">
+      <c r="Q54" s="19">
         <v>46030</v>
       </c>
-      <c r="Q54"/>
       <c r="R54"/>
-    </row>
-    <row r="55" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S54"/>
+    </row>
+    <row r="55" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>113</v>
       </c>
@@ -3698,32 +3863,35 @@
       <c r="H55" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="I55" s="13" t="s">
+      <c r="I55" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J55" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K55" s="18" t="s">
+      <c r="K55" s="17" t="s">
         <v>241</v>
       </c>
-      <c r="L55" s="15"/>
-      <c r="M55" s="4">
+      <c r="L55" s="14"/>
+      <c r="M55" s="19">
         <v>46063</v>
       </c>
-      <c r="N55" s="7" t="s">
+      <c r="N55" s="4">
+        <v>46063</v>
+      </c>
+      <c r="O55" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="O55" s="20">
+      <c r="P55" s="19">
         <v>46063</v>
       </c>
-      <c r="P55" s="20">
+      <c r="Q55" s="19">
         <v>46063</v>
       </c>
-      <c r="Q55"/>
       <c r="R55"/>
-    </row>
-    <row r="56" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S55"/>
+    </row>
+    <row r="56" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>113</v>
       </c>
@@ -3746,32 +3914,35 @@
       <c r="H56" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="I56" s="13" t="s">
+      <c r="I56" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J56" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K56" s="18" t="s">
+      <c r="K56" s="17" t="s">
         <v>241</v>
       </c>
-      <c r="L56" s="15"/>
-      <c r="M56" s="4">
+      <c r="L56" s="14"/>
+      <c r="M56" s="19">
         <v>46204</v>
       </c>
-      <c r="N56" s="7" t="s">
+      <c r="N56" s="4">
+        <v>46204</v>
+      </c>
+      <c r="O56" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="O56" s="20">
+      <c r="P56" s="19">
         <v>46204</v>
       </c>
-      <c r="P56" s="20">
+      <c r="Q56" s="19">
         <v>46204</v>
       </c>
-      <c r="Q56"/>
       <c r="R56"/>
-    </row>
-    <row r="57" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S56"/>
+    </row>
+    <row r="57" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
         <v>113</v>
       </c>
@@ -3794,32 +3965,35 @@
       <c r="H57" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="I57" s="13" t="s">
+      <c r="I57" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J57" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K57" s="18" t="s">
+      <c r="K57" s="17" t="s">
         <v>241</v>
       </c>
-      <c r="L57" s="15"/>
-      <c r="M57" s="4">
+      <c r="L57" s="14"/>
+      <c r="M57" s="19">
         <v>46209</v>
       </c>
-      <c r="N57" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="O57" s="20">
+      <c r="N57" s="4">
         <v>46209</v>
       </c>
-      <c r="P57" s="20">
+      <c r="O57" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="P57" s="19">
         <v>46209</v>
       </c>
-      <c r="Q57"/>
+      <c r="Q57" s="19">
+        <v>46209</v>
+      </c>
       <c r="R57"/>
-    </row>
-    <row r="58" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S57"/>
+    </row>
+    <row r="58" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>113</v>
       </c>
@@ -3842,32 +4016,35 @@
       <c r="H58" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="I58" s="13" t="s">
+      <c r="I58" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J58" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K58" s="18" t="s">
+      <c r="K58" s="17" t="s">
         <v>241</v>
       </c>
-      <c r="L58" s="15"/>
-      <c r="M58" s="4">
+      <c r="L58" s="14"/>
+      <c r="M58" s="19">
         <v>46220</v>
       </c>
-      <c r="N58" s="7" t="s">
+      <c r="N58" s="4">
+        <v>46220</v>
+      </c>
+      <c r="O58" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="O58" s="20">
+      <c r="P58" s="19">
         <v>46220</v>
       </c>
-      <c r="P58" s="20">
+      <c r="Q58" s="19">
         <v>46220</v>
       </c>
-      <c r="Q58"/>
       <c r="R58"/>
-    </row>
-    <row r="59" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S58"/>
+    </row>
+    <row r="59" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>133</v>
       </c>
@@ -3890,32 +4067,35 @@
       <c r="H59" s="8" t="s">
         <v>234</v>
       </c>
-      <c r="I59" s="13" t="s">
+      <c r="I59" s="12" t="s">
         <v>235</v>
       </c>
       <c r="J59" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K59" s="18" t="s">
+      <c r="K59" s="17" t="s">
         <v>240</v>
       </c>
-      <c r="L59" s="15"/>
-      <c r="M59" s="4">
+      <c r="L59" s="14"/>
+      <c r="M59" s="19">
         <v>46217</v>
       </c>
-      <c r="N59" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="O59" s="20">
+      <c r="N59" s="4">
         <v>46217</v>
       </c>
-      <c r="P59" s="20">
+      <c r="O59" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="P59" s="19">
         <v>46217</v>
       </c>
-      <c r="Q59"/>
+      <c r="Q59" s="19">
+        <v>46217</v>
+      </c>
       <c r="R59"/>
-    </row>
-    <row r="60" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S59"/>
+    </row>
+    <row r="60" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>133</v>
       </c>
@@ -3938,32 +4118,35 @@
       <c r="H60" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="I60" s="13" t="s">
+      <c r="I60" s="12" t="s">
         <v>233</v>
       </c>
       <c r="J60" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K60" s="18" t="s">
+      <c r="K60" s="17" t="s">
         <v>236</v>
       </c>
-      <c r="L60" s="15"/>
-      <c r="M60" s="4">
+      <c r="L60" s="14"/>
+      <c r="M60" s="19">
         <v>46223</v>
       </c>
-      <c r="N60" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="O60" s="20">
+      <c r="N60" s="4">
         <v>46223</v>
       </c>
-      <c r="P60" s="20">
+      <c r="O60" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="P60" s="19">
         <v>46223</v>
       </c>
-      <c r="Q60"/>
+      <c r="Q60" s="19">
+        <v>46223</v>
+      </c>
       <c r="R60"/>
-    </row>
-    <row r="61" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S60"/>
+    </row>
+    <row r="61" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>133</v>
       </c>
@@ -3983,35 +4166,38 @@
       <c r="G61" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="H61" s="9" t="s">
+      <c r="H61" s="8" t="s">
         <v>223</v>
       </c>
-      <c r="I61" s="13" t="s">
+      <c r="I61" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J61" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K61" s="18" t="s">
+      <c r="K61" s="17" t="s">
         <v>236</v>
       </c>
-      <c r="L61" s="15"/>
-      <c r="M61" s="4">
+      <c r="L61" s="14"/>
+      <c r="M61" s="19">
         <v>46224</v>
       </c>
-      <c r="N61" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="O61" s="20">
+      <c r="N61" s="4">
         <v>46224</v>
       </c>
-      <c r="P61" s="20">
+      <c r="O61" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="P61" s="19">
         <v>46224</v>
       </c>
-      <c r="Q61"/>
+      <c r="Q61" s="19">
+        <v>46224</v>
+      </c>
       <c r="R61"/>
-    </row>
-    <row r="62" spans="1:18" ht="12.75" hidden="1" x14ac:dyDescent="0.2">
+      <c r="S61"/>
+    </row>
+    <row r="62" spans="1:19" ht="12.75" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>133</v>
       </c>
@@ -4034,39 +4220,36 @@
       <c r="H62" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="I62" s="13" t="s">
+      <c r="I62" s="12" t="s">
         <v>232</v>
       </c>
       <c r="J62" s="7" t="s">
         <v>215</v>
       </c>
-      <c r="K62" s="18" t="s">
+      <c r="K62" s="17" t="s">
         <v>237</v>
       </c>
-      <c r="L62" s="15"/>
-      <c r="M62" s="4">
+      <c r="L62" s="14"/>
+      <c r="M62" s="19">
         <v>46226</v>
       </c>
-      <c r="N62" s="7" t="s">
-        <v>220</v>
-      </c>
-      <c r="O62" s="20">
+      <c r="N62" s="4">
         <v>46226</v>
       </c>
-      <c r="P62" s="20">
+      <c r="O62" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="P62" s="19">
         <v>46226</v>
       </c>
-      <c r="Q62"/>
+      <c r="Q62" s="19">
+        <v>46226</v>
+      </c>
       <c r="R62"/>
+      <c r="S62"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R62" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="1">
-      <filters>
-        <filter val="Enjoy Pucón"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:S62" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -4121,72 +4304,72 @@
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A14" s="11" t="s">
+      <c r="A14" s="10" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="10" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A16" s="11" t="s">
+      <c r="A16" s="10" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="11" t="s">
+      <c r="A17" s="10" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" s="11" t="s">
+      <c r="A18" s="10" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="10" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="10" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" s="12" t="s">
+      <c r="A21" s="11" t="s">
         <v>211</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" s="12" t="s">
+      <c r="A22" s="11" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="11" t="s">
         <v>219</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="10" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="10" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="10" t="s">
         <v>147</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="10" t="s">
         <v>148</v>
       </c>
     </row>

</xml_diff>